<commit_message>
huge renaming update to new canonical titles
</commit_message>
<xml_diff>
--- a/PKSim/Analog10_PKSim.xlsx
+++ b/PKSim/Analog10_PKSim.xlsx
@@ -6,7 +6,7 @@
     <workbookView tabRatio="600"/>
   </bookViews>
   <sheets>
-    <sheet name="Analog10_PKSim" sheetId="1" r:id="rId3"/>
+    <sheet name="Analog11_PKSim" sheetId="1" r:id="rId3"/>
     <sheet name="Global PK-Analyses" sheetId="2" r:id="rId4"/>
     <sheet name="PK-Analyses" sheetId="3" r:id="rId5"/>
   </sheets>
@@ -19,16 +19,16 @@
     <t xml:space="preserve">Time [h]</t>
   </si>
   <si>
-    <t xml:space="preserve">Analog10-Peripheral Venous Blood-Plasma-Concentration [µmol/l]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10-Arterial Blood-Plasma-Concentration [µmol/l]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10-Brain-Tissue-Concentration [µmol/l]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10-Liver-Tissue-Concentration [µmol/l]</t>
+    <t xml:space="preserve">Analog11-Peripheral Venous Blood-Plasma-Concentration [µmol/l]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11-Arterial Blood-Plasma-Concentration [µmol/l]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11-Brain-Tissue-Concentration [µmol/l]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11-Liver-Tissue-Concentration [µmol/l]</t>
   </si>
   <si>
     <t xml:space="preserve">Parameter</t>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Vss (plasma)</t>
   </si>
   <si>
-    <t xml:space="preserve">Analog10</t>
+    <t xml:space="preserve">Analog11</t>
   </si>
   <si>
     <t xml:space="preserve">ml/kg</t>
@@ -64,16 +64,16 @@
     <t xml:space="preserve">Vss (phys-chem)</t>
   </si>
   <si>
-    <t xml:space="preserve">Analog10 - Analog10-Arterial Blood-Plasma-Concentration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10 - Analog10-Brain-Tissue-Concentration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10 - Analog10-Liver-Tissue-Concentration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analog10 - Analog10-Peripheral Venous Blood-Plasma-Concentration</t>
+    <t xml:space="preserve">Analog11 - Analog11-Arterial Blood-Plasma-Concentration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11 - Analog11-Brain-Tissue-Concentration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11 - Analog11-Liver-Tissue-Concentration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analog11 - Analog11-Peripheral Venous Blood-Plasma-Concentration</t>
   </si>
   <si>
     <t xml:space="preserve">AUC_inf [µmol*min/l]</t>
@@ -173,10 +173,10 @@
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.55" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="65.1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.85" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.95" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.55" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -218,16 +218,16 @@
         <v>0.05</v>
       </c>
       <c r="B3" s="2">
-        <v>0.001490698</v>
+        <v>0.001514583</v>
       </c>
       <c r="C3" s="2">
-        <v>0.001166836</v>
+        <v>0.001184391</v>
       </c>
       <c r="D3" s="2">
-        <v>3.05737E-06</v>
+        <v>3.126104E-06</v>
       </c>
       <c r="E3" s="2">
-        <v>0.001506795</v>
+        <v>0.001571987</v>
       </c>
     </row>
     <row r="4">
@@ -235,16 +235,16 @@
         <v>0.1</v>
       </c>
       <c r="B4" s="2">
-        <v>0.001021768</v>
+        <v>0.0010333</v>
       </c>
       <c r="C4" s="2">
-        <v>0.0008470261</v>
+        <v>0.0008673533</v>
       </c>
       <c r="D4" s="2">
-        <v>2.242899E-06</v>
+        <v>2.418633E-06</v>
       </c>
       <c r="E4" s="2">
-        <v>0.001916331</v>
+        <v>0.001949607</v>
       </c>
     </row>
     <row r="5">
@@ -252,16 +252,16 @@
         <v>0.15</v>
       </c>
       <c r="B5" s="2">
-        <v>0.0007927016</v>
+        <v>0.0008067627</v>
       </c>
       <c r="C5" s="2">
-        <v>0.0007369178</v>
+        <v>0.0007575966</v>
       </c>
       <c r="D5" s="2">
-        <v>2.198494E-06</v>
+        <v>2.419073E-06</v>
       </c>
       <c r="E5" s="2">
-        <v>0.001882438</v>
+        <v>0.00187685</v>
       </c>
     </row>
     <row r="6">
@@ -269,16 +269,16 @@
         <v>0.2</v>
       </c>
       <c r="B6" s="2">
-        <v>0.0006770687</v>
+        <v>0.0006922068</v>
       </c>
       <c r="C6" s="2">
-        <v>0.0006623933</v>
+        <v>0.0006798337</v>
       </c>
       <c r="D6" s="2">
-        <v>2.229961E-06</v>
+        <v>2.475695E-06</v>
       </c>
       <c r="E6" s="2">
-        <v>0.001726393</v>
+        <v>0.001697329</v>
       </c>
     </row>
     <row r="7">
@@ -286,16 +286,16 @@
         <v>0.25</v>
       </c>
       <c r="B7" s="2">
-        <v>0.0006055182</v>
+        <v>0.0006198413</v>
       </c>
       <c r="C7" s="2">
-        <v>0.0006015059</v>
+        <v>0.0006155439</v>
       </c>
       <c r="D7" s="2">
-        <v>2.272882E-06</v>
+        <v>2.538489E-06</v>
       </c>
       <c r="E7" s="2">
-        <v>0.001554366</v>
+        <v>0.001514141</v>
       </c>
     </row>
     <row r="8">
@@ -303,16 +303,16 @@
         <v>0.3</v>
       </c>
       <c r="B8" s="2">
-        <v>0.0005527959</v>
+        <v>0.0005657986</v>
       </c>
       <c r="C8" s="2">
-        <v>0.0005497456</v>
+        <v>0.0005611906</v>
       </c>
       <c r="D8" s="2">
-        <v>2.318422E-06</v>
+        <v>2.602095E-06</v>
       </c>
       <c r="E8" s="2">
-        <v>0.001397106</v>
+        <v>0.001352779</v>
       </c>
     </row>
     <row r="9">
@@ -320,16 +320,16 @@
         <v>0.35</v>
       </c>
       <c r="B9" s="2">
-        <v>0.0005100867</v>
+        <v>0.0005219514</v>
       </c>
       <c r="C9" s="2">
-        <v>0.000505394</v>
+        <v>0.0005151021</v>
       </c>
       <c r="D9" s="2">
-        <v>2.365059E-06</v>
+        <v>2.665905E-06</v>
       </c>
       <c r="E9" s="2">
-        <v>0.001260966</v>
+        <v>0.001216247</v>
       </c>
     </row>
     <row r="10">
@@ -337,16 +337,16 @@
         <v>0.4</v>
       </c>
       <c r="B10" s="2">
-        <v>0.0004740388</v>
+        <v>0.000485112</v>
       </c>
       <c r="C10" s="2">
-        <v>0.0004672848</v>
+        <v>0.0004759239</v>
       </c>
       <c r="D10" s="2">
-        <v>2.412369E-06</v>
+        <v>2.72973E-06</v>
       </c>
       <c r="E10" s="2">
-        <v>0.001144932</v>
+        <v>0.001101736</v>
       </c>
     </row>
     <row r="11">
@@ -354,16 +354,16 @@
         <v>0.45</v>
       </c>
       <c r="B11" s="2">
-        <v>0.0004430895</v>
+        <v>0.0004536853</v>
       </c>
       <c r="C11" s="2">
-        <v>0.0004344338</v>
+        <v>0.0004424757</v>
       </c>
       <c r="D11" s="2">
-        <v>2.460089E-06</v>
+        <v>2.793337E-06</v>
       </c>
       <c r="E11" s="2">
-        <v>0.001046186</v>
+        <v>0.001005499</v>
       </c>
     </row>
     <row r="12">
@@ -371,16 +371,16 @@
         <v>0.5</v>
       </c>
       <c r="B12" s="2">
-        <v>0.0004162352</v>
+        <v>0.0004266133</v>
       </c>
       <c r="C12" s="2">
-        <v>0.0004059958</v>
+        <v>0.0004137631</v>
       </c>
       <c r="D12" s="2">
-        <v>2.507962E-06</v>
+        <v>2.856497E-06</v>
       </c>
       <c r="E12" s="2">
-        <v>0.0009619453</v>
+        <v>0.0009242081</v>
       </c>
     </row>
     <row r="13">
@@ -388,16 +388,16 @@
         <v>0.55</v>
       </c>
       <c r="B13" s="2">
-        <v>0.000392797</v>
+        <v>0.0004031126</v>
       </c>
       <c r="C13" s="2">
-        <v>0.000381267</v>
+        <v>0.0003889676</v>
       </c>
       <c r="D13" s="2">
-        <v>2.555782E-06</v>
+        <v>2.919019E-06</v>
       </c>
       <c r="E13" s="2">
-        <v>0.0008897172</v>
+        <v>0.0008551236</v>
       </c>
     </row>
     <row r="14">
@@ -405,16 +405,16 @@
         <v>0.6</v>
       </c>
       <c r="B14" s="2">
-        <v>0.0003722282</v>
+        <v>0.0003825575</v>
       </c>
       <c r="C14" s="2">
-        <v>0.0003596577</v>
+        <v>0.0003674214</v>
       </c>
       <c r="D14" s="2">
-        <v>2.603378E-06</v>
+        <v>2.980761E-06</v>
       </c>
       <c r="E14" s="2">
-        <v>0.0008274584</v>
+        <v>0.0007960587</v>
       </c>
     </row>
     <row r="15">
@@ -422,16 +422,16 @@
         <v>0.65</v>
       </c>
       <c r="B15" s="2">
-        <v>0.0003540632</v>
+        <v>0.0003644553</v>
       </c>
       <c r="C15" s="2">
-        <v>0.0003406793</v>
+        <v>0.0003485837</v>
       </c>
       <c r="D15" s="2">
-        <v>2.650615E-06</v>
+        <v>3.041627E-06</v>
       </c>
       <c r="E15" s="2">
-        <v>0.0007735373</v>
+        <v>0.0007452457</v>
       </c>
     </row>
     <row r="16">
@@ -439,16 +439,16 @@
         <v>0.7</v>
       </c>
       <c r="B16" s="2">
-        <v>0.0003379337</v>
+        <v>0.0003484077</v>
       </c>
       <c r="C16" s="2">
-        <v>0.0003239288</v>
+        <v>0.0003320118</v>
       </c>
       <c r="D16" s="2">
-        <v>2.697396E-06</v>
+        <v>3.101553E-06</v>
       </c>
       <c r="E16" s="2">
-        <v>0.0007266007</v>
+        <v>0.0007012633</v>
       </c>
     </row>
     <row r="17">
@@ -456,16 +456,16 @@
         <v>0.75</v>
       </c>
       <c r="B17" s="2">
-        <v>0.0003235337</v>
+        <v>0.0003340848</v>
       </c>
       <c r="C17" s="2">
-        <v>0.00030907</v>
+        <v>0.0003173422</v>
       </c>
       <c r="D17" s="2">
-        <v>2.74365E-06</v>
+        <v>3.160495E-06</v>
       </c>
       <c r="E17" s="2">
-        <v>0.0006855403</v>
+        <v>0.0006629701</v>
       </c>
     </row>
     <row r="18">
@@ -473,16 +473,16 @@
         <v>0.8</v>
       </c>
       <c r="B18" s="2">
-        <v>0.0003106082</v>
+        <v>0.0003212147</v>
       </c>
       <c r="C18" s="2">
-        <v>0.0002958236</v>
+        <v>0.0003042756</v>
       </c>
       <c r="D18" s="2">
-        <v>2.789324E-06</v>
+        <v>3.218426E-06</v>
       </c>
       <c r="E18" s="2">
-        <v>0.0006494488</v>
+        <v>0.0006294348</v>
       </c>
     </row>
     <row r="19">
@@ -490,16 +490,16 @@
         <v>0.85</v>
       </c>
       <c r="B19" s="2">
-        <v>0.0002989435</v>
+        <v>0.0003095763</v>
       </c>
       <c r="C19" s="2">
-        <v>0.000283956</v>
+        <v>0.0002925651</v>
       </c>
       <c r="D19" s="2">
-        <v>2.83438E-06</v>
+        <v>3.275335E-06</v>
       </c>
       <c r="E19" s="2">
-        <v>0.0006175757</v>
+        <v>0.0005998877</v>
       </c>
     </row>
     <row r="20">
@@ -507,16 +507,16 @@
         <v>0.9</v>
       </c>
       <c r="B20" s="2">
-        <v>0.0002883617</v>
+        <v>0.0002989904</v>
       </c>
       <c r="C20" s="2">
-        <v>0.0002732709</v>
+        <v>0.0002820068</v>
       </c>
       <c r="D20" s="2">
-        <v>2.878794E-06</v>
+        <v>3.331223E-06</v>
       </c>
       <c r="E20" s="2">
-        <v>0.0005892934</v>
+        <v>0.0005736933</v>
       </c>
     </row>
     <row r="21">
@@ -524,16 +524,16 @@
         <v>0.95</v>
       </c>
       <c r="B21" s="2">
-        <v>0.0002787136</v>
+        <v>0.0002893073</v>
       </c>
       <c r="C21" s="2">
-        <v>0.0002636027</v>
+        <v>0.0002724313</v>
       </c>
       <c r="D21" s="2">
-        <v>2.92255E-06</v>
+        <v>3.386093E-06</v>
       </c>
       <c r="E21" s="2">
-        <v>0.0005640741</v>
+        <v>0.0005503304</v>
       </c>
     </row>
     <row r="22">
@@ -541,16 +541,16 @@
         <v>1</v>
       </c>
       <c r="B22" s="2">
-        <v>0.0002698737</v>
+        <v>0.0002804013</v>
       </c>
       <c r="C22" s="2">
-        <v>0.0002548113</v>
+        <v>0.0002636977</v>
       </c>
       <c r="D22" s="2">
-        <v>2.965638E-06</v>
+        <v>3.439956E-06</v>
       </c>
       <c r="E22" s="2">
-        <v>0.0005414751</v>
+        <v>0.0005293711</v>
       </c>
     </row>
     <row r="23">
@@ -558,16 +558,16 @@
         <v>1.05</v>
       </c>
       <c r="B23" s="2">
-        <v>0.0002617359</v>
+        <v>0.0002721659</v>
       </c>
       <c r="C23" s="2">
-        <v>0.0002467787</v>
+        <v>0.0002556876</v>
       </c>
       <c r="D23" s="2">
-        <v>3.008052E-06</v>
+        <v>3.492824E-06</v>
       </c>
       <c r="E23" s="2">
-        <v>0.000521125</v>
+        <v>0.0005104587</v>
       </c>
     </row>
     <row r="24">
@@ -575,16 +575,16 @@
         <v>1.1</v>
       </c>
       <c r="B24" s="2">
-        <v>0.0002542096</v>
+        <v>0.000264515</v>
       </c>
       <c r="C24" s="2">
-        <v>0.0002394043</v>
+        <v>0.0002483035</v>
       </c>
       <c r="D24" s="2">
-        <v>3.049794E-06</v>
+        <v>3.544714E-06</v>
       </c>
       <c r="E24" s="2">
-        <v>0.0005027093</v>
+        <v>0.0004932963</v>
       </c>
     </row>
     <row r="25">
@@ -592,16 +592,16 @@
         <v>1.15</v>
       </c>
       <c r="B25" s="2">
-        <v>0.0002472186</v>
+        <v>0.0002573708</v>
       </c>
       <c r="C25" s="2">
-        <v>0.0002326031</v>
+        <v>0.0002414601</v>
       </c>
       <c r="D25" s="2">
-        <v>3.090866E-06</v>
+        <v>3.595644E-06</v>
       </c>
       <c r="E25" s="2">
-        <v>0.0004859632</v>
+        <v>0.0004776308</v>
       </c>
     </row>
     <row r="26">
@@ -609,16 +609,16 @@
         <v>1.2</v>
       </c>
       <c r="B26" s="2">
-        <v>0.0002406977</v>
+        <v>0.0002506734</v>
       </c>
       <c r="C26" s="2">
-        <v>0.0002263025</v>
+        <v>0.0002350887</v>
       </c>
       <c r="D26" s="2">
-        <v>3.131274E-06</v>
+        <v>3.645633E-06</v>
       </c>
       <c r="E26" s="2">
-        <v>0.000470661</v>
+        <v>0.0004632521</v>
       </c>
     </row>
     <row r="27">
@@ -626,16 +626,16 @@
         <v>1.25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.0002345926</v>
+        <v>0.0002443704</v>
       </c>
       <c r="C27" s="2">
-        <v>0.0002204421</v>
+        <v>0.0002291303</v>
       </c>
       <c r="D27" s="2">
-        <v>3.171025E-06</v>
+        <v>3.694703E-06</v>
       </c>
       <c r="E27" s="2">
-        <v>0.0004566161</v>
+        <v>0.0004499839</v>
       </c>
     </row>
     <row r="28">
@@ -643,16 +643,16 @@
         <v>1.3</v>
       </c>
       <c r="B28" s="2">
-        <v>0.000228856</v>
+        <v>0.0002384182</v>
       </c>
       <c r="C28" s="2">
-        <v>0.0002149694</v>
+        <v>0.0002235353</v>
       </c>
       <c r="D28" s="2">
-        <v>3.210128E-06</v>
+        <v>3.742875E-06</v>
       </c>
       <c r="E28" s="2">
-        <v>0.000443667</v>
+        <v>0.000437678</v>
       </c>
     </row>
     <row r="29">
@@ -660,16 +660,16 @@
         <v>1.35</v>
       </c>
       <c r="B29" s="2">
-        <v>0.0002234474</v>
+        <v>0.0002327798</v>
       </c>
       <c r="C29" s="2">
-        <v>0.0002098393</v>
+        <v>0.0002182626</v>
       </c>
       <c r="D29" s="2">
-        <v>3.248595E-06</v>
+        <v>3.79017E-06</v>
       </c>
       <c r="E29" s="2">
-        <v>0.0004316752</v>
+        <v>0.0004262138</v>
       </c>
     </row>
     <row r="30">
@@ -677,16 +677,16 @@
         <v>1.4</v>
       </c>
       <c r="B30" s="2">
-        <v>0.0002183318</v>
+        <v>0.0002274234</v>
       </c>
       <c r="C30" s="2">
-        <v>0.0002050132</v>
+        <v>0.0002132771</v>
       </c>
       <c r="D30" s="2">
-        <v>3.286435E-06</v>
+        <v>3.836612E-06</v>
       </c>
       <c r="E30" s="2">
-        <v>0.0004205227</v>
+        <v>0.0004154887</v>
       </c>
     </row>
     <row r="31">
@@ -694,16 +694,16 @@
         <v>1.45</v>
       </c>
       <c r="B31" s="2">
-        <v>0.0002134788</v>
+        <v>0.0002223216</v>
       </c>
       <c r="C31" s="2">
-        <v>0.0002004574</v>
+        <v>0.0002085489</v>
       </c>
       <c r="D31" s="2">
-        <v>3.323662E-06</v>
+        <v>3.882221E-06</v>
       </c>
       <c r="E31" s="2">
-        <v>0.000410107</v>
+        <v>0.0004054159</v>
       </c>
     </row>
     <row r="32">
@@ -711,16 +711,16 @@
         <v>1.5</v>
       </c>
       <c r="B32" s="2">
-        <v>0.0002088628</v>
+        <v>0.0002174512</v>
       </c>
       <c r="C32" s="2">
-        <v>0.0001961437</v>
+        <v>0.0002040525</v>
       </c>
       <c r="D32" s="2">
-        <v>3.360287E-06</v>
+        <v>3.92702E-06</v>
       </c>
       <c r="E32" s="2">
-        <v>0.0004003425</v>
+        <v>0.0003959213</v>
       </c>
     </row>
     <row r="33">
@@ -728,16 +728,16 @@
         <v>1.55</v>
       </c>
       <c r="B33" s="2">
-        <v>0.0002044616</v>
+        <v>0.000212792</v>
       </c>
       <c r="C33" s="2">
-        <v>0.0001920477</v>
+        <v>0.0001997657</v>
       </c>
       <c r="D33" s="2">
-        <v>3.396322E-06</v>
+        <v>3.971031E-06</v>
       </c>
       <c r="E33" s="2">
-        <v>0.0003911559</v>
+        <v>0.0003869408</v>
       </c>
     </row>
     <row r="34">
@@ -745,16 +745,16 @@
         <v>1.6</v>
       </c>
       <c r="B34" s="2">
-        <v>0.0002002562</v>
+        <v>0.000208327</v>
       </c>
       <c r="C34" s="2">
-        <v>0.0001881487</v>
+        <v>0.0001956697</v>
       </c>
       <c r="D34" s="2">
-        <v>3.431782E-06</v>
+        <v>4.014275E-06</v>
       </c>
       <c r="E34" s="2">
-        <v>0.0003824849</v>
+        <v>0.0003784202</v>
       </c>
     </row>
     <row r="35">
@@ -762,16 +762,16 @@
         <v>1.65</v>
       </c>
       <c r="B35" s="2">
-        <v>0.0001962301</v>
+        <v>0.0002040414</v>
       </c>
       <c r="C35" s="2">
-        <v>0.0001844284</v>
+        <v>0.0001917483</v>
       </c>
       <c r="D35" s="2">
-        <v>3.466679E-06</v>
+        <v>4.056772E-06</v>
       </c>
       <c r="E35" s="2">
-        <v>0.0003742759</v>
+        <v>0.0003703141</v>
       </c>
     </row>
     <row r="36">
@@ -779,16 +779,16 @@
         <v>1.7</v>
       </c>
       <c r="B36" s="2">
-        <v>0.000192369</v>
+        <v>0.0001999221</v>
       </c>
       <c r="C36" s="2">
-        <v>0.0001808717</v>
+        <v>0.0001879877</v>
       </c>
       <c r="D36" s="2">
-        <v>3.501026E-06</v>
+        <v>4.098545E-06</v>
       </c>
       <c r="E36" s="2">
-        <v>0.0003664837</v>
+        <v>0.0003625835</v>
       </c>
     </row>
     <row r="37">
@@ -796,16 +796,16 @@
         <v>1.75</v>
       </c>
       <c r="B37" s="2">
-        <v>0.0001886602</v>
+        <v>0.0001959578</v>
       </c>
       <c r="C37" s="2">
-        <v>0.0001774646</v>
+        <v>0.0001843759</v>
       </c>
       <c r="D37" s="2">
-        <v>3.534837E-06</v>
+        <v>4.139614E-06</v>
       </c>
       <c r="E37" s="2">
-        <v>0.0003590673</v>
+        <v>0.0003551958</v>
       </c>
     </row>
     <row r="38">
@@ -813,16 +813,16 @@
         <v>1.8</v>
       </c>
       <c r="B38" s="2">
-        <v>0.0001850927</v>
+        <v>0.0001921386</v>
       </c>
       <c r="C38" s="2">
-        <v>0.0001741953</v>
+        <v>0.0001809024</v>
       </c>
       <c r="D38" s="2">
-        <v>3.568125E-06</v>
+        <v>4.179998E-06</v>
       </c>
       <c r="E38" s="2">
-        <v>0.0003519925</v>
+        <v>0.0003481224</v>
       </c>
     </row>
     <row r="39">
@@ -830,16 +830,16 @@
         <v>1.85</v>
       </c>
       <c r="B39" s="2">
-        <v>0.0001816569</v>
+        <v>0.0001884557</v>
       </c>
       <c r="C39" s="2">
-        <v>0.0001710537</v>
+        <v>0.0001775579</v>
       </c>
       <c r="D39" s="2">
-        <v>3.600903E-06</v>
+        <v>4.219716E-06</v>
       </c>
       <c r="E39" s="2">
-        <v>0.00034523</v>
+        <v>0.0003413384</v>
       </c>
     </row>
     <row r="40">
@@ -847,16 +847,16 @@
         <v>1.9</v>
       </c>
       <c r="B40" s="2">
-        <v>0.0001783431</v>
+        <v>0.0001849013</v>
       </c>
       <c r="C40" s="2">
-        <v>0.0001680292</v>
+        <v>0.0001743344</v>
       </c>
       <c r="D40" s="2">
-        <v>3.633183E-06</v>
+        <v>4.258789E-06</v>
       </c>
       <c r="E40" s="2">
-        <v>0.0003387495</v>
+        <v>0.0003348218</v>
       </c>
     </row>
     <row r="41">
@@ -864,16 +864,16 @@
         <v>1.95</v>
       </c>
       <c r="B41" s="2">
-        <v>0.0001751451</v>
+        <v>0.0001814686</v>
       </c>
       <c r="C41" s="2">
-        <v>0.0001651155</v>
+        <v>0.0001712247</v>
       </c>
       <c r="D41" s="2">
-        <v>3.664978E-06</v>
+        <v>4.297234E-06</v>
       </c>
       <c r="E41" s="2">
-        <v>0.0003325331</v>
+        <v>0.0003285537</v>
       </c>
     </row>
     <row r="42">
@@ -881,16 +881,16 @@
         <v>2</v>
       </c>
       <c r="B42" s="2">
-        <v>0.0001720547</v>
+        <v>0.0001781512</v>
       </c>
       <c r="C42" s="2">
-        <v>0.000162304</v>
+        <v>0.0001682223</v>
       </c>
       <c r="D42" s="2">
-        <v>3.696301E-06</v>
+        <v>4.33507E-06</v>
       </c>
       <c r="E42" s="2">
-        <v>0.0003265563</v>
+        <v>0.0003225174</v>
       </c>
     </row>
     <row r="43">
@@ -898,16 +898,16 @@
         <v>2.25</v>
       </c>
       <c r="B43" s="2">
-        <v>0.0001580326</v>
+        <v>0.0001631145</v>
       </c>
       <c r="C43" s="2">
-        <v>0.0001495877</v>
+        <v>0.0001546399</v>
       </c>
       <c r="D43" s="2">
-        <v>3.846245E-06</v>
+        <v>4.515708E-06</v>
       </c>
       <c r="E43" s="2">
-        <v>0.0002997474</v>
+        <v>0.0002953655</v>
       </c>
     </row>
     <row r="44">
@@ -915,16 +915,16 @@
         <v>2.5</v>
       </c>
       <c r="B44" s="2">
-        <v>0.000146025</v>
+        <v>0.0001502926</v>
       </c>
       <c r="C44" s="2">
-        <v>0.000138735</v>
+        <v>0.0001430793</v>
       </c>
       <c r="D44" s="2">
-        <v>3.986108E-06</v>
+        <v>4.683557E-06</v>
       </c>
       <c r="E44" s="2">
-        <v>0.0002770848</v>
+        <v>0.000272396</v>
       </c>
     </row>
     <row r="45">
@@ -932,16 +932,16 @@
         <v>2.75</v>
       </c>
       <c r="B45" s="2">
-        <v>0.0001356632</v>
+        <v>0.0001393035</v>
       </c>
       <c r="C45" s="2">
-        <v>0.000129384</v>
+        <v>0.0001331756</v>
       </c>
       <c r="D45" s="2">
-        <v>4.117162E-06</v>
+        <v>4.840372E-06</v>
       </c>
       <c r="E45" s="2">
-        <v>0.0002576614</v>
+        <v>0.0002527793</v>
       </c>
     </row>
     <row r="46">
@@ -949,16 +949,16 @@
         <v>3</v>
       </c>
       <c r="B46" s="2">
-        <v>0.0001266778</v>
+        <v>0.00012986</v>
       </c>
       <c r="C46" s="2">
-        <v>0.0001212781</v>
+        <v>0.0001246634</v>
       </c>
       <c r="D46" s="2">
-        <v>4.240524E-06</v>
+        <v>4.987663E-06</v>
       </c>
       <c r="E46" s="2">
-        <v>0.0002408689</v>
+        <v>0.000235949</v>
       </c>
     </row>
     <row r="47">
@@ -966,16 +966,16 @@
         <v>3.25</v>
       </c>
       <c r="B47" s="2">
-        <v>0.0001188644</v>
+        <v>0.0001217307</v>
       </c>
       <c r="C47" s="2">
-        <v>0.0001142274</v>
+        <v>0.000117332</v>
       </c>
       <c r="D47" s="2">
-        <v>4.357169E-06</v>
+        <v>5.126727E-06</v>
       </c>
       <c r="E47" s="2">
-        <v>0.0002262826</v>
+        <v>0.0002214707</v>
       </c>
     </row>
     <row r="48">
@@ -983,16 +983,16 @@
         <v>3.5</v>
       </c>
       <c r="B48" s="2">
-        <v>0.0001120629</v>
+        <v>0.0001147215</v>
       </c>
       <c r="C48" s="2">
-        <v>0.0001080871</v>
+        <v>0.0001110054</v>
       </c>
       <c r="D48" s="2">
-        <v>4.467946E-06</v>
+        <v>5.258676E-06</v>
       </c>
       <c r="E48" s="2">
-        <v>0.0002135951</v>
+        <v>0.0002089869</v>
       </c>
     </row>
     <row r="49">
@@ -1000,16 +1000,16 @@
         <v>3.75</v>
       </c>
       <c r="B49" s="2">
-        <v>0.0001061343</v>
+        <v>0.0001086691</v>
       </c>
       <c r="C49" s="2">
-        <v>0.0001027313</v>
+        <v>0.0001055366</v>
       </c>
       <c r="D49" s="2">
-        <v>4.573591E-06</v>
+        <v>5.384465E-06</v>
       </c>
       <c r="E49" s="2">
-        <v>0.0002025386</v>
+        <v>0.0001982014</v>
       </c>
     </row>
     <row r="50">
@@ -1017,16 +1017,16 @@
         <v>4</v>
       </c>
       <c r="B50" s="2">
-        <v>0.0001009591</v>
+        <v>0.0001034377</v>
       </c>
       <c r="C50" s="2">
-        <v>9.805156E-05</v>
+        <v>0.0001008039</v>
       </c>
       <c r="D50" s="2">
-        <v>4.674741E-06</v>
+        <v>5.504912E-06</v>
       </c>
       <c r="E50" s="2">
-        <v>0.0001928839</v>
+        <v>0.0001888743</v>
       </c>
     </row>
     <row r="51">
@@ -1034,16 +1034,16 @@
         <v>4.25</v>
       </c>
       <c r="B51" s="2">
-        <v>9.643698E-05</v>
+        <v>9.891096E-05</v>
       </c>
       <c r="C51" s="2">
-        <v>9.395825E-05</v>
+        <v>9.670365E-05</v>
       </c>
       <c r="D51" s="2">
-        <v>4.771952E-06</v>
+        <v>5.620719E-06</v>
       </c>
       <c r="E51" s="2">
-        <v>0.0001844448</v>
+        <v>0.0001808008</v>
       </c>
     </row>
     <row r="52">
@@ -1051,16 +1051,16 @@
         <v>4.5</v>
       </c>
       <c r="B52" s="2">
-        <v>9.248137E-05</v>
+        <v>9.498783E-05</v>
       </c>
       <c r="C52" s="2">
-        <v>9.037356E-05</v>
+        <v>9.31449E-05</v>
       </c>
       <c r="D52" s="2">
-        <v>4.865706E-06</v>
+        <v>5.732489E-06</v>
       </c>
       <c r="E52" s="2">
-        <v>0.0001770601</v>
+        <v>0.0001738001</v>
       </c>
     </row>
     <row r="53">
@@ -1068,16 +1068,16 @@
         <v>4.75</v>
       </c>
       <c r="B53" s="2">
-        <v>8.901636E-05</v>
+        <v>9.158163E-05</v>
       </c>
       <c r="C53" s="2">
-        <v>8.722932E-05</v>
+        <v>9.004984E-05</v>
       </c>
       <c r="D53" s="2">
-        <v>4.956418E-06</v>
+        <v>5.840737E-06</v>
       </c>
       <c r="E53" s="2">
-        <v>0.0001705874</v>
+        <v>0.0001677168</v>
       </c>
     </row>
     <row r="54">
@@ -1085,16 +1085,16 @@
         <v>5</v>
       </c>
       <c r="B54" s="2">
-        <v>8.597679E-05</v>
+        <v>8.86191E-05</v>
       </c>
       <c r="C54" s="2">
-        <v>8.446704E-05</v>
+        <v>8.735291E-05</v>
       </c>
       <c r="D54" s="2">
-        <v>5.044452E-06</v>
+        <v>5.945908E-06</v>
       </c>
       <c r="E54" s="2">
-        <v>0.0001649055</v>
+        <v>0.0001624213</v>
       </c>
     </row>
     <row r="55">
@@ -1102,16 +1102,16 @@
         <v>5.25</v>
       </c>
       <c r="B55" s="2">
-        <v>8.330628E-05</v>
+        <v>8.603765E-05</v>
       </c>
       <c r="C55" s="2">
-        <v>8.203621E-05</v>
+        <v>8.499817E-05</v>
       </c>
       <c r="D55" s="2">
-        <v>5.130124E-06</v>
+        <v>6.048382E-06</v>
       </c>
       <c r="E55" s="2">
-        <v>0.0001599098</v>
+        <v>0.0001578033</v>
       </c>
     </row>
     <row r="56">
@@ -1119,16 +1119,16 @@
         <v>5.5</v>
       </c>
       <c r="B56" s="2">
-        <v>8.095604E-05</v>
+        <v>8.378318E-05</v>
       </c>
       <c r="C56" s="2">
-        <v>7.989311E-05</v>
+        <v>8.293707E-05</v>
       </c>
       <c r="D56" s="2">
-        <v>5.213706E-06</v>
+        <v>6.148487E-06</v>
       </c>
       <c r="E56" s="2">
-        <v>0.0001555097</v>
+        <v>0.0001537663</v>
       </c>
     </row>
     <row r="57">
@@ -1136,16 +1136,16 @@
         <v>5.75</v>
       </c>
       <c r="B57" s="2">
-        <v>7.888434E-05</v>
+        <v>8.18093E-05</v>
       </c>
       <c r="C57" s="2">
-        <v>7.800041E-05</v>
+        <v>8.1128E-05</v>
       </c>
       <c r="D57" s="2">
-        <v>5.295436E-06</v>
+        <v>6.246503E-06</v>
       </c>
       <c r="E57" s="2">
-        <v>0.0001516282</v>
+        <v>0.0001502277</v>
       </c>
     </row>
     <row r="58">
@@ -1153,16 +1153,16 @@
         <v>6</v>
       </c>
       <c r="B58" s="2">
-        <v>7.705452E-05</v>
+        <v>8.007648E-05</v>
       </c>
       <c r="C58" s="2">
-        <v>7.632517E-05</v>
+        <v>7.953557E-05</v>
       </c>
       <c r="D58" s="2">
-        <v>5.375518E-06</v>
+        <v>6.342672E-06</v>
       </c>
       <c r="E58" s="2">
-        <v>0.0001481969</v>
+        <v>0.0001471173</v>
       </c>
     </row>
     <row r="59">
@@ -1170,16 +1170,16 @@
         <v>6.25</v>
       </c>
       <c r="B59" s="2">
-        <v>7.543475E-05</v>
+        <v>7.855085E-05</v>
       </c>
       <c r="C59" s="2">
-        <v>7.48388E-05</v>
+        <v>7.812942E-05</v>
       </c>
       <c r="D59" s="2">
-        <v>5.454132E-06</v>
+        <v>6.437203E-06</v>
       </c>
       <c r="E59" s="2">
-        <v>0.0001451563</v>
+        <v>0.000144375</v>
       </c>
     </row>
     <row r="60">
@@ -1187,16 +1187,16 @@
         <v>6.5</v>
       </c>
       <c r="B60" s="2">
-        <v>7.399741E-05</v>
+        <v>7.720365E-05</v>
       </c>
       <c r="C60" s="2">
-        <v>7.351657E-05</v>
+        <v>7.688381E-05</v>
       </c>
       <c r="D60" s="2">
-        <v>5.531435E-06</v>
+        <v>6.530274E-06</v>
       </c>
       <c r="E60" s="2">
-        <v>0.0001424552</v>
+        <v>0.00014195</v>
       </c>
     </row>
     <row r="61">
@@ -1204,16 +1204,16 @@
         <v>6.75</v>
       </c>
       <c r="B61" s="2">
-        <v>7.271879E-05</v>
+        <v>7.600997E-05</v>
       </c>
       <c r="C61" s="2">
-        <v>7.233716E-05</v>
+        <v>7.577643E-05</v>
       </c>
       <c r="D61" s="2">
-        <v>5.607562E-06</v>
+        <v>6.62204E-06</v>
       </c>
       <c r="E61" s="2">
-        <v>0.0001400493</v>
+        <v>0.0001397981</v>
       </c>
     </row>
     <row r="62">
@@ -1221,16 +1221,16 @@
         <v>7</v>
       </c>
       <c r="B62" s="2">
-        <v>7.157821E-05</v>
+        <v>7.494861E-05</v>
       </c>
       <c r="C62" s="2">
-        <v>7.128207E-05</v>
+        <v>7.47883E-05</v>
       </c>
       <c r="D62" s="2">
-        <v>5.682632E-06</v>
+        <v>6.712634E-06</v>
       </c>
       <c r="E62" s="2">
-        <v>0.0001379003</v>
+        <v>0.0001378818</v>
       </c>
     </row>
     <row r="63">
@@ -1238,16 +1238,16 @@
         <v>7.25</v>
       </c>
       <c r="B63" s="2">
-        <v>7.055778E-05</v>
+        <v>7.400123E-05</v>
       </c>
       <c r="C63" s="2">
-        <v>7.033526E-05</v>
+        <v>7.390301E-05</v>
       </c>
       <c r="D63" s="2">
-        <v>5.756747E-06</v>
+        <v>6.802172E-06</v>
       </c>
       <c r="E63" s="2">
-        <v>0.0001359751</v>
+        <v>0.0001361687</v>
       </c>
     </row>
     <row r="64">
@@ -1255,16 +1255,16 @@
         <v>7.5</v>
       </c>
       <c r="B64" s="2">
-        <v>6.964197E-05</v>
+        <v>7.315211E-05</v>
       </c>
       <c r="C64" s="2">
-        <v>6.948279E-05</v>
+        <v>7.310643E-05</v>
       </c>
       <c r="D64" s="2">
-        <v>5.829999E-06</v>
+        <v>6.890753E-06</v>
       </c>
       <c r="E64" s="2">
-        <v>0.0001342449</v>
+        <v>0.0001346307</v>
       </c>
     </row>
     <row r="65">
@@ -1272,16 +1272,16 @@
         <v>7.75</v>
       </c>
       <c r="B65" s="2">
-        <v>6.88174E-05</v>
+        <v>7.238761E-05</v>
       </c>
       <c r="C65" s="2">
-        <v>6.871267E-05</v>
+        <v>7.238632E-05</v>
       </c>
       <c r="D65" s="2">
-        <v>5.902466E-06</v>
+        <v>6.978465E-06</v>
       </c>
       <c r="E65" s="2">
-        <v>0.0001326846</v>
+        <v>0.0001332435</v>
       </c>
     </row>
     <row r="66">
@@ -1289,16 +1289,16 @@
         <v>8</v>
       </c>
       <c r="B66" s="2">
-        <v>6.807242E-05</v>
+        <v>7.169632E-05</v>
       </c>
       <c r="C66" s="2">
-        <v>6.801441E-05</v>
+        <v>7.173241E-05</v>
       </c>
       <c r="D66" s="2">
-        <v>5.974216E-06</v>
+        <v>7.065381E-06</v>
       </c>
       <c r="E66" s="2">
-        <v>0.0001312728</v>
+        <v>0.0001319866</v>
       </c>
     </row>
     <row r="67">
@@ -1306,16 +1306,16 @@
         <v>8.25</v>
       </c>
       <c r="B67" s="2">
-        <v>6.739688E-05</v>
+        <v>7.106835E-05</v>
       </c>
       <c r="C67" s="2">
-        <v>6.737896E-05</v>
+        <v>7.113585E-05</v>
       </c>
       <c r="D67" s="2">
-        <v>6.04531E-06</v>
+        <v>7.151565E-06</v>
       </c>
       <c r="E67" s="2">
-        <v>0.0001299904</v>
+        <v>0.0001308424</v>
       </c>
     </row>
     <row r="68">
@@ -1323,16 +1323,16 @@
         <v>8.5</v>
       </c>
       <c r="B68" s="2">
-        <v>6.678203E-05</v>
+        <v>7.049541E-05</v>
       </c>
       <c r="C68" s="2">
-        <v>6.679842E-05</v>
+        <v>7.058919E-05</v>
       </c>
       <c r="D68" s="2">
-        <v>6.1158E-06</v>
+        <v>7.237074E-06</v>
       </c>
       <c r="E68" s="2">
-        <v>0.0001288212</v>
+        <v>0.0001297963</v>
       </c>
     </row>
     <row r="69">
@@ -1340,16 +1340,16 @@
         <v>8.75</v>
       </c>
       <c r="B69" s="2">
-        <v>6.622017E-05</v>
+        <v>6.997031E-05</v>
       </c>
       <c r="C69" s="2">
-        <v>6.626589E-05</v>
+        <v>7.008601E-05</v>
       </c>
       <c r="D69" s="2">
-        <v>6.185733E-06</v>
+        <v>7.321957E-06</v>
       </c>
       <c r="E69" s="2">
-        <v>0.000127751</v>
+        <v>0.0001288356</v>
       </c>
     </row>
     <row r="70">
@@ -1357,16 +1357,16 @@
         <v>9</v>
       </c>
       <c r="B70" s="2">
-        <v>6.570479E-05</v>
+        <v>6.948688E-05</v>
       </c>
       <c r="C70" s="2">
-        <v>6.577554E-05</v>
+        <v>6.962079E-05</v>
       </c>
       <c r="D70" s="2">
-        <v>6.255149E-06</v>
+        <v>7.406256E-06</v>
       </c>
       <c r="E70" s="2">
-        <v>0.0001267676</v>
+        <v>0.0001279495</v>
       </c>
     </row>
     <row r="71">
@@ -1374,16 +1374,16 @@
         <v>9.25</v>
       </c>
       <c r="B71" s="2">
-        <v>6.523012E-05</v>
+        <v>6.903976E-05</v>
       </c>
       <c r="C71" s="2">
-        <v>6.532217E-05</v>
+        <v>6.918871E-05</v>
       </c>
       <c r="D71" s="2">
-        <v>6.324085E-06</v>
+        <v>7.490009E-06</v>
       </c>
       <c r="E71" s="2">
-        <v>0.0001258603</v>
+        <v>0.0001271284</v>
       </c>
     </row>
     <row r="72">
@@ -1391,16 +1391,16 @@
         <v>9.5</v>
       </c>
       <c r="B72" s="2">
-        <v>6.479127E-05</v>
+        <v>6.862434E-05</v>
       </c>
       <c r="C72" s="2">
-        <v>6.490142E-05</v>
+        <v>6.878562E-05</v>
       </c>
       <c r="D72" s="2">
-        <v>6.392572E-06</v>
+        <v>7.573251E-06</v>
       </c>
       <c r="E72" s="2">
-        <v>0.0001250199</v>
+        <v>0.0001263641</v>
       </c>
     </row>
     <row r="73">
@@ -1408,16 +1408,16 @@
         <v>9.75</v>
       </c>
       <c r="B73" s="2">
-        <v>6.43841E-05</v>
+        <v>6.823662E-05</v>
       </c>
       <c r="C73" s="2">
-        <v>6.450952E-05</v>
+        <v>6.840791E-05</v>
       </c>
       <c r="D73" s="2">
-        <v>6.460636E-06</v>
+        <v>7.656008E-06</v>
       </c>
       <c r="E73" s="2">
-        <v>0.0001242389</v>
+        <v>0.0001256495</v>
       </c>
     </row>
     <row r="74">
@@ -1425,16 +1425,16 @@
         <v>10</v>
       </c>
       <c r="B74" s="2">
-        <v>6.400477E-05</v>
+        <v>6.787325E-05</v>
       </c>
       <c r="C74" s="2">
-        <v>6.414306E-05</v>
+        <v>6.805259E-05</v>
       </c>
       <c r="D74" s="2">
-        <v>6.528302E-06</v>
+        <v>7.738308E-06</v>
       </c>
       <c r="E74" s="2">
-        <v>0.00012351</v>
+        <v>0.0001249784</v>
       </c>
     </row>
     <row r="75">
@@ -1442,16 +1442,16 @@
         <v>10.25</v>
       </c>
       <c r="B75" s="2">
-        <v>6.365019E-05</v>
+        <v>6.753133E-05</v>
       </c>
       <c r="C75" s="2">
-        <v>6.379925E-05</v>
+        <v>6.771703E-05</v>
       </c>
       <c r="D75" s="2">
-        <v>6.595593E-06</v>
+        <v>7.820173E-06</v>
       </c>
       <c r="E75" s="2">
-        <v>0.0001228276</v>
+        <v>0.0001243459</v>
       </c>
     </row>
     <row r="76">
@@ -1459,16 +1459,16 @@
         <v>10.5</v>
       </c>
       <c r="B76" s="2">
-        <v>6.331743E-05</v>
+        <v>6.720838E-05</v>
       </c>
       <c r="C76" s="2">
-        <v>6.347545E-05</v>
+        <v>6.739903E-05</v>
       </c>
       <c r="D76" s="2">
-        <v>6.662527E-06</v>
+        <v>7.901622E-06</v>
       </c>
       <c r="E76" s="2">
-        <v>0.000122186</v>
+        <v>0.0001237476</v>
       </c>
     </row>
     <row r="77">
@@ -1476,16 +1476,16 @@
         <v>10.75</v>
       </c>
       <c r="B77" s="2">
-        <v>6.300398E-05</v>
+        <v>6.690233E-05</v>
       </c>
       <c r="C77" s="2">
-        <v>6.316941E-05</v>
+        <v>6.709668E-05</v>
       </c>
       <c r="D77" s="2">
-        <v>6.729122E-06</v>
+        <v>7.982674E-06</v>
       </c>
       <c r="E77" s="2">
-        <v>0.0001215808</v>
+        <v>0.0001231796</v>
       </c>
     </row>
     <row r="78">
@@ -1493,16 +1493,16 @@
         <v>11</v>
       </c>
       <c r="B78" s="2">
-        <v>6.270773E-05</v>
+        <v>6.66113E-05</v>
       </c>
       <c r="C78" s="2">
-        <v>6.287923E-05</v>
+        <v>6.680833E-05</v>
       </c>
       <c r="D78" s="2">
-        <v>6.795395E-06</v>
+        <v>8.063345E-06</v>
       </c>
       <c r="E78" s="2">
-        <v>0.0001210079</v>
+        <v>0.0001226388</v>
       </c>
     </row>
     <row r="79">
@@ -1510,16 +1510,16 @@
         <v>11.25</v>
       </c>
       <c r="B79" s="2">
-        <v>6.242668E-05</v>
+        <v>6.633369E-05</v>
       </c>
       <c r="C79" s="2">
-        <v>6.26031E-05</v>
+        <v>6.653252E-05</v>
       </c>
       <c r="D79" s="2">
-        <v>6.861359E-06</v>
+        <v>8.14365E-06</v>
       </c>
       <c r="E79" s="2">
-        <v>0.0001204636</v>
+        <v>0.0001221223</v>
       </c>
     </row>
     <row r="80">
@@ -1527,16 +1527,16 @@
         <v>11.5</v>
       </c>
       <c r="B80" s="2">
-        <v>6.215928E-05</v>
+        <v>6.606823E-05</v>
       </c>
       <c r="C80" s="2">
-        <v>6.233963E-05</v>
+        <v>6.62681E-05</v>
       </c>
       <c r="D80" s="2">
-        <v>6.927027E-06</v>
+        <v>8.223601E-06</v>
       </c>
       <c r="E80" s="2">
-        <v>0.0001199451</v>
+        <v>0.0001216277</v>
       </c>
     </row>
     <row r="81">
@@ -1544,16 +1544,16 @@
         <v>11.75</v>
       </c>
       <c r="B81" s="2">
-        <v>6.190409E-05</v>
+        <v>6.581369E-05</v>
       </c>
       <c r="C81" s="2">
-        <v>6.208752E-05</v>
+        <v>6.601396E-05</v>
       </c>
       <c r="D81" s="2">
-        <v>6.99241E-06</v>
+        <v>8.30321E-06</v>
       </c>
       <c r="E81" s="2">
-        <v>0.0001194496</v>
+        <v>0.0001211529</v>
       </c>
     </row>
     <row r="82">
@@ -1561,16 +1561,16 @@
         <v>12</v>
       </c>
       <c r="B82" s="2">
-        <v>6.165991E-05</v>
+        <v>6.556884E-05</v>
       </c>
       <c r="C82" s="2">
-        <v>6.184569E-05</v>
+        <v>6.576902E-05</v>
       </c>
       <c r="D82" s="2">
-        <v>7.057519E-06</v>
+        <v>8.38249E-06</v>
       </c>
       <c r="E82" s="2">
-        <v>0.0001189749</v>
+        <v>0.0001206959</v>
       </c>
     </row>
     <row r="83">
@@ -1578,16 +1578,16 @@
         <v>12.25</v>
       </c>
       <c r="B83" s="2">
-        <v>6.142571E-05</v>
+        <v>6.533296E-05</v>
       </c>
       <c r="C83" s="2">
-        <v>6.16132E-05</v>
+        <v>6.553259E-05</v>
       </c>
       <c r="D83" s="2">
-        <v>7.122363E-06</v>
+        <v>8.461449E-06</v>
       </c>
       <c r="E83" s="2">
-        <v>0.0001185192</v>
+        <v>0.0001202552</v>
       </c>
     </row>
     <row r="84">
@@ -1595,16 +1595,16 @@
         <v>12.5</v>
       </c>
       <c r="B84" s="2">
-        <v>6.120055E-05</v>
+        <v>6.510527E-05</v>
       </c>
       <c r="C84" s="2">
-        <v>6.138921E-05</v>
+        <v>6.530397E-05</v>
       </c>
       <c r="D84" s="2">
-        <v>7.18695E-06</v>
+        <v>8.540098E-06</v>
       </c>
       <c r="E84" s="2">
-        <v>0.0001180806</v>
+        <v>0.0001198294</v>
       </c>
     </row>
     <row r="85">
@@ -1612,16 +1612,16 @@
         <v>12.75</v>
       </c>
       <c r="B85" s="2">
-        <v>6.098364E-05</v>
+        <v>6.488481E-05</v>
       </c>
       <c r="C85" s="2">
-        <v>6.117301E-05</v>
+        <v>6.508231E-05</v>
       </c>
       <c r="D85" s="2">
-        <v>7.251288E-06</v>
+        <v>8.618445E-06</v>
       </c>
       <c r="E85" s="2">
-        <v>0.0001176576</v>
+        <v>0.000119417</v>
       </c>
     </row>
     <row r="86">
@@ -1629,16 +1629,16 @@
         <v>13</v>
       </c>
       <c r="B86" s="2">
-        <v>6.077427E-05</v>
+        <v>6.467109E-05</v>
       </c>
       <c r="C86" s="2">
-        <v>6.096394E-05</v>
+        <v>6.486716E-05</v>
       </c>
       <c r="D86" s="2">
-        <v>7.315385E-06</v>
+        <v>8.696499E-06</v>
       </c>
       <c r="E86" s="2">
-        <v>0.0001172491</v>
+        <v>0.000119017</v>
       </c>
     </row>
     <row r="87">
@@ -1646,16 +1646,16 @@
         <v>13.25</v>
       </c>
       <c r="B87" s="2">
-        <v>6.057187E-05</v>
+        <v>6.446373E-05</v>
       </c>
       <c r="C87" s="2">
-        <v>6.07615E-05</v>
+        <v>6.465813E-05</v>
       </c>
       <c r="D87" s="2">
-        <v>7.379246E-06</v>
+        <v>8.774266E-06</v>
       </c>
       <c r="E87" s="2">
-        <v>0.0001168538</v>
+        <v>0.0001186286</v>
       </c>
     </row>
     <row r="88">
@@ -1663,16 +1663,16 @@
         <v>13.5</v>
       </c>
       <c r="B88" s="2">
-        <v>6.037587E-05</v>
+        <v>6.426209E-05</v>
       </c>
       <c r="C88" s="2">
-        <v>6.056515E-05</v>
+        <v>6.445467E-05</v>
       </c>
       <c r="D88" s="2">
-        <v>7.442878E-06</v>
+        <v>8.851755E-06</v>
       </c>
       <c r="E88" s="2">
-        <v>0.0001164707</v>
+        <v>0.0001182507</v>
       </c>
     </row>
     <row r="89">
@@ -1680,16 +1680,16 @@
         <v>13.75</v>
       </c>
       <c r="B89" s="2">
-        <v>6.018573E-05</v>
+        <v>6.40658E-05</v>
       </c>
       <c r="C89" s="2">
-        <v>6.037442E-05</v>
+        <v>6.425643E-05</v>
       </c>
       <c r="D89" s="2">
-        <v>7.506288E-06</v>
+        <v>8.92897E-06</v>
       </c>
       <c r="E89" s="2">
-        <v>0.0001160988</v>
+        <v>0.0001178828</v>
       </c>
     </row>
     <row r="90">
@@ -1697,16 +1697,16 @@
         <v>14</v>
       </c>
       <c r="B90" s="2">
-        <v>6.000104E-05</v>
+        <v>6.387467E-05</v>
       </c>
       <c r="C90" s="2">
-        <v>6.018893E-05</v>
+        <v>6.406323E-05</v>
       </c>
       <c r="D90" s="2">
-        <v>7.56948E-06</v>
+        <v>9.005918E-06</v>
       </c>
       <c r="E90" s="2">
-        <v>0.0001157374</v>
+        <v>0.0001175243</v>
       </c>
     </row>
     <row r="91">
@@ -1714,16 +1714,16 @@
         <v>14.25</v>
       </c>
       <c r="B91" s="2">
-        <v>5.982152E-05</v>
+        <v>6.368835E-05</v>
       </c>
       <c r="C91" s="2">
-        <v>6.000842E-05</v>
+        <v>6.387474E-05</v>
       </c>
       <c r="D91" s="2">
-        <v>7.63246E-06</v>
+        <v>9.082605E-06</v>
       </c>
       <c r="E91" s="2">
-        <v>0.0001153859</v>
+        <v>0.0001171746</v>
       </c>
     </row>
     <row r="92">
@@ -1731,16 +1731,16 @@
         <v>14.5</v>
       </c>
       <c r="B92" s="2">
-        <v>5.964669E-05</v>
+        <v>6.35066E-05</v>
       </c>
       <c r="C92" s="2">
-        <v>5.983246E-05</v>
+        <v>6.369076E-05</v>
       </c>
       <c r="D92" s="2">
-        <v>7.695231E-06</v>
+        <v>9.159035E-06</v>
       </c>
       <c r="E92" s="2">
-        <v>0.0001150434</v>
+        <v>0.0001168334</v>
       </c>
     </row>
     <row r="93">
@@ -1748,16 +1748,16 @@
         <v>14.75</v>
       </c>
       <c r="B93" s="2">
-        <v>5.947622E-05</v>
+        <v>6.332923E-05</v>
       </c>
       <c r="C93" s="2">
-        <v>5.966073E-05</v>
+        <v>6.351109E-05</v>
       </c>
       <c r="D93" s="2">
-        <v>7.757801E-06</v>
+        <v>9.235216E-06</v>
       </c>
       <c r="E93" s="2">
-        <v>0.0001147093</v>
+        <v>0.0001165003</v>
       </c>
     </row>
     <row r="94">
@@ -1765,16 +1765,16 @@
         <v>15</v>
       </c>
       <c r="B94" s="2">
-        <v>5.931002E-05</v>
+        <v>6.315605E-05</v>
       </c>
       <c r="C94" s="2">
-        <v>5.949316E-05</v>
+        <v>6.333556E-05</v>
       </c>
       <c r="D94" s="2">
-        <v>7.820171E-06</v>
+        <v>9.31115E-06</v>
       </c>
       <c r="E94" s="2">
-        <v>0.0001143834</v>
+        <v>0.0001161749</v>
       </c>
     </row>
     <row r="95">
@@ -1782,16 +1782,16 @@
         <v>15.25</v>
       </c>
       <c r="B95" s="2">
-        <v>5.914774E-05</v>
+        <v>6.298688E-05</v>
       </c>
       <c r="C95" s="2">
-        <v>5.932943E-05</v>
+        <v>6.316401E-05</v>
       </c>
       <c r="D95" s="2">
-        <v>7.882347E-06</v>
+        <v>9.386844E-06</v>
       </c>
       <c r="E95" s="2">
-        <v>0.0001140652</v>
+        <v>0.0001158571</v>
       </c>
     </row>
     <row r="96">
@@ -1799,16 +1799,16 @@
         <v>15.5</v>
       </c>
       <c r="B96" s="2">
-        <v>5.898913E-05</v>
+        <v>6.282159E-05</v>
       </c>
       <c r="C96" s="2">
-        <v>5.91693E-05</v>
+        <v>6.29963E-05</v>
       </c>
       <c r="D96" s="2">
-        <v>7.944333E-06</v>
+        <v>9.462301E-06</v>
       </c>
       <c r="E96" s="2">
-        <v>0.000113754</v>
+        <v>0.0001155464</v>
       </c>
     </row>
     <row r="97">
@@ -1816,16 +1816,16 @@
         <v>15.75</v>
       </c>
       <c r="B97" s="2">
-        <v>5.883411E-05</v>
+        <v>6.265997E-05</v>
       </c>
       <c r="C97" s="2">
-        <v>5.90127E-05</v>
+        <v>6.283227E-05</v>
       </c>
       <c r="D97" s="2">
-        <v>8.006131E-06</v>
+        <v>9.537525E-06</v>
       </c>
       <c r="E97" s="2">
-        <v>0.0001134497</v>
+        <v>0.0001152425</v>
       </c>
     </row>
     <row r="98">
@@ -1833,16 +1833,16 @@
         <v>16</v>
       </c>
       <c r="B98" s="2">
-        <v>5.868247E-05</v>
+        <v>6.250185E-05</v>
       </c>
       <c r="C98" s="2">
-        <v>5.885944E-05</v>
+        <v>6.267172E-05</v>
       </c>
       <c r="D98" s="2">
-        <v>8.067746E-06</v>
+        <v>9.612524E-06</v>
       </c>
       <c r="E98" s="2">
-        <v>0.000113152</v>
+        <v>0.0001149452</v>
       </c>
     </row>
     <row r="99">
@@ -1850,16 +1850,16 @@
         <v>16.25</v>
       </c>
       <c r="B99" s="2">
-        <v>5.853408E-05</v>
+        <v>6.234711E-05</v>
       </c>
       <c r="C99" s="2">
-        <v>5.87094E-05</v>
+        <v>6.251457E-05</v>
       </c>
       <c r="D99" s="2">
-        <v>8.129182E-06</v>
+        <v>9.687299E-06</v>
       </c>
       <c r="E99" s="2">
-        <v>0.0001128606</v>
+        <v>0.0001146543</v>
       </c>
     </row>
     <row r="100">
@@ -1867,16 +1867,16 @@
         <v>16.5</v>
       </c>
       <c r="B100" s="2">
-        <v>5.838881E-05</v>
+        <v>6.219575E-05</v>
       </c>
       <c r="C100" s="2">
-        <v>5.856244E-05</v>
+        <v>6.236078E-05</v>
       </c>
       <c r="D100" s="2">
-        <v>8.190441E-06</v>
+        <v>9.761855E-06</v>
       </c>
       <c r="E100" s="2">
-        <v>0.0001125753</v>
+        <v>0.0001143696</v>
       </c>
     </row>
     <row r="101">
@@ -1884,16 +1884,16 @@
         <v>16.75</v>
       </c>
       <c r="B101" s="2">
-        <v>5.824654E-05</v>
+        <v>6.204752E-05</v>
       </c>
       <c r="C101" s="2">
-        <v>5.841847E-05</v>
+        <v>6.221014E-05</v>
       </c>
       <c r="D101" s="2">
-        <v>8.251526E-06</v>
+        <v>9.836195E-06</v>
       </c>
       <c r="E101" s="2">
-        <v>0.0001122959</v>
+        <v>0.0001140908</v>
       </c>
     </row>
     <row r="102">
@@ -1901,16 +1901,16 @@
         <v>17</v>
       </c>
       <c r="B102" s="2">
-        <v>5.810718E-05</v>
+        <v>6.190224E-05</v>
       </c>
       <c r="C102" s="2">
-        <v>5.827739E-05</v>
+        <v>6.206249E-05</v>
       </c>
       <c r="D102" s="2">
-        <v>8.312441E-06</v>
+        <v>9.910325E-06</v>
       </c>
       <c r="E102" s="2">
-        <v>0.000112022</v>
+        <v>0.0001138175</v>
       </c>
     </row>
     <row r="103">
@@ -1918,16 +1918,16 @@
         <v>17.25</v>
       </c>
       <c r="B103" s="2">
-        <v>5.797063E-05</v>
+        <v>6.175985E-05</v>
       </c>
       <c r="C103" s="2">
-        <v>5.81391E-05</v>
+        <v>6.191774E-05</v>
       </c>
       <c r="D103" s="2">
-        <v>8.373189E-06</v>
+        <v>9.984249E-06</v>
       </c>
       <c r="E103" s="2">
-        <v>0.0001117537</v>
+        <v>0.0001135497</v>
       </c>
     </row>
     <row r="104">
@@ -1935,16 +1935,16 @@
         <v>17.5</v>
       </c>
       <c r="B104" s="2">
-        <v>5.783681E-05</v>
+        <v>6.16204E-05</v>
       </c>
       <c r="C104" s="2">
-        <v>5.800353E-05</v>
+        <v>6.177594E-05</v>
       </c>
       <c r="D104" s="2">
-        <v>8.433773E-06</v>
+        <v>1.005797E-05</v>
       </c>
       <c r="E104" s="2">
-        <v>0.0001114906</v>
+        <v>0.0001132873</v>
       </c>
     </row>
     <row r="105">
@@ -1952,16 +1952,16 @@
         <v>17.75</v>
       </c>
       <c r="B105" s="2">
-        <v>5.770561E-05</v>
+        <v>6.148368E-05</v>
       </c>
       <c r="C105" s="2">
-        <v>5.787058E-05</v>
+        <v>6.163692E-05</v>
       </c>
       <c r="D105" s="2">
-        <v>8.494194E-06</v>
+        <v>1.013149E-05</v>
       </c>
       <c r="E105" s="2">
-        <v>0.0001112327</v>
+        <v>0.0001130301</v>
       </c>
     </row>
     <row r="106">
@@ -1969,16 +1969,16 @@
         <v>18</v>
       </c>
       <c r="B106" s="2">
-        <v>5.757694E-05</v>
+        <v>6.134961E-05</v>
       </c>
       <c r="C106" s="2">
-        <v>5.774017E-05</v>
+        <v>6.150057E-05</v>
       </c>
       <c r="D106" s="2">
-        <v>8.554456E-06</v>
+        <v>1.020481E-05</v>
       </c>
       <c r="E106" s="2">
-        <v>0.0001109797</v>
+        <v>0.0001127778</v>
       </c>
     </row>
     <row r="107">
@@ -1986,16 +1986,16 @@
         <v>18.25</v>
       </c>
       <c r="B107" s="2">
-        <v>5.745072E-05</v>
+        <v>6.121812E-05</v>
       </c>
       <c r="C107" s="2">
-        <v>5.761221E-05</v>
+        <v>6.136683E-05</v>
       </c>
       <c r="D107" s="2">
-        <v>8.614563E-06</v>
+        <v>1.027794E-05</v>
       </c>
       <c r="E107" s="2">
-        <v>0.0001107315</v>
+        <v>0.0001125303</v>
       </c>
     </row>
     <row r="108">
@@ -2003,16 +2003,16 @@
         <v>18.5</v>
       </c>
       <c r="B108" s="2">
-        <v>5.732694E-05</v>
+        <v>6.108921E-05</v>
       </c>
       <c r="C108" s="2">
-        <v>5.748669E-05</v>
+        <v>6.123571E-05</v>
       </c>
       <c r="D108" s="2">
-        <v>8.674515E-06</v>
+        <v>1.035088E-05</v>
       </c>
       <c r="E108" s="2">
-        <v>0.0001104881</v>
+        <v>0.0001122877</v>
       </c>
     </row>
     <row r="109">
@@ -2020,16 +2020,16 @@
         <v>18.75</v>
       </c>
       <c r="B109" s="2">
-        <v>5.720548E-05</v>
+        <v>6.09628E-05</v>
       </c>
       <c r="C109" s="2">
-        <v>5.736351E-05</v>
+        <v>6.110712E-05</v>
       </c>
       <c r="D109" s="2">
-        <v>8.734317E-06</v>
+        <v>1.042364E-05</v>
       </c>
       <c r="E109" s="2">
-        <v>0.0001102492</v>
+        <v>0.0001120498</v>
       </c>
     </row>
     <row r="110">
@@ -2037,16 +2037,16 @@
         <v>19</v>
       </c>
       <c r="B110" s="2">
-        <v>5.708625E-05</v>
+        <v>6.083886E-05</v>
       </c>
       <c r="C110" s="2">
-        <v>5.724257E-05</v>
+        <v>6.098101E-05</v>
       </c>
       <c r="D110" s="2">
-        <v>8.79397E-06</v>
+        <v>1.049621E-05</v>
       </c>
       <c r="E110" s="2">
-        <v>0.0001100146</v>
+        <v>0.0001118164</v>
       </c>
     </row>
     <row r="111">
@@ -2054,16 +2054,16 @@
         <v>19.25</v>
       </c>
       <c r="B111" s="2">
-        <v>5.696921E-05</v>
+        <v>6.071732E-05</v>
       </c>
       <c r="C111" s="2">
-        <v>5.712383E-05</v>
+        <v>6.085735E-05</v>
       </c>
       <c r="D111" s="2">
-        <v>8.853477E-06</v>
+        <v>1.05686E-05</v>
       </c>
       <c r="E111" s="2">
-        <v>0.0001097844</v>
+        <v>0.0001115877</v>
       </c>
     </row>
     <row r="112">
@@ -2071,16 +2071,16 @@
         <v>19.5</v>
       </c>
       <c r="B112" s="2">
-        <v>5.685434E-05</v>
+        <v>6.059812E-05</v>
       </c>
       <c r="C112" s="2">
-        <v>5.700728E-05</v>
+        <v>6.073605E-05</v>
       </c>
       <c r="D112" s="2">
-        <v>8.912841E-06</v>
+        <v>1.064081E-05</v>
       </c>
       <c r="E112" s="2">
-        <v>0.0001095584</v>
+        <v>0.0001113632</v>
       </c>
     </row>
     <row r="113">
@@ -2088,16 +2088,16 @@
         <v>19.75</v>
       </c>
       <c r="B113" s="2">
-        <v>5.674158E-05</v>
+        <v>6.048124E-05</v>
       </c>
       <c r="C113" s="2">
-        <v>5.689284E-05</v>
+        <v>6.061709E-05</v>
       </c>
       <c r="D113" s="2">
-        <v>8.972062E-06</v>
+        <v>1.071285E-05</v>
       </c>
       <c r="E113" s="2">
-        <v>0.0001093365</v>
+        <v>0.0001111432</v>
       </c>
     </row>
     <row r="114">
@@ -2105,16 +2105,16 @@
         <v>20</v>
       </c>
       <c r="B114" s="2">
-        <v>5.663085E-05</v>
+        <v>6.036663E-05</v>
       </c>
       <c r="C114" s="2">
-        <v>5.678046E-05</v>
+        <v>6.050045E-05</v>
       </c>
       <c r="D114" s="2">
-        <v>9.031145E-06</v>
+        <v>1.078471E-05</v>
       </c>
       <c r="E114" s="2">
-        <v>0.0001091186</v>
+        <v>0.0001109274</v>
       </c>
     </row>
     <row r="115">
@@ -2122,16 +2122,16 @@
         <v>20.25</v>
       </c>
       <c r="B115" s="2">
-        <v>5.652212E-05</v>
+        <v>6.025425E-05</v>
       </c>
       <c r="C115" s="2">
-        <v>5.66701E-05</v>
+        <v>6.038605E-05</v>
       </c>
       <c r="D115" s="2">
-        <v>9.090091E-06</v>
+        <v>1.085641E-05</v>
       </c>
       <c r="E115" s="2">
-        <v>0.0001089046</v>
+        <v>0.0001107158</v>
       </c>
     </row>
     <row r="116">
@@ -2139,16 +2139,16 @@
         <v>20.5</v>
       </c>
       <c r="B116" s="2">
-        <v>5.641537E-05</v>
+        <v>6.014404E-05</v>
       </c>
       <c r="C116" s="2">
-        <v>5.656173E-05</v>
+        <v>6.027385E-05</v>
       </c>
       <c r="D116" s="2">
-        <v>9.148903E-06</v>
+        <v>1.092794E-05</v>
       </c>
       <c r="E116" s="2">
-        <v>0.0001086945</v>
+        <v>0.0001105083</v>
       </c>
     </row>
     <row r="117">
@@ -2156,16 +2156,16 @@
         <v>20.75</v>
       </c>
       <c r="B117" s="2">
-        <v>5.631056E-05</v>
+        <v>6.003594E-05</v>
       </c>
       <c r="C117" s="2">
-        <v>5.645532E-05</v>
+        <v>6.01638E-05</v>
       </c>
       <c r="D117" s="2">
-        <v>9.207581E-06</v>
+        <v>1.09993E-05</v>
       </c>
       <c r="E117" s="2">
-        <v>0.0001084882</v>
+        <v>0.0001103047</v>
       </c>
     </row>
     <row r="118">
@@ -2173,16 +2173,16 @@
         <v>21</v>
       </c>
       <c r="B118" s="2">
-        <v>5.620765E-05</v>
+        <v>5.992991E-05</v>
       </c>
       <c r="C118" s="2">
-        <v>5.635082E-05</v>
+        <v>6.005584E-05</v>
       </c>
       <c r="D118" s="2">
-        <v>9.266128E-06</v>
+        <v>1.107051E-05</v>
       </c>
       <c r="E118" s="2">
-        <v>0.0001082856</v>
+        <v>0.000110105</v>
       </c>
     </row>
     <row r="119">
@@ -2190,16 +2190,16 @@
         <v>21.25</v>
       </c>
       <c r="B119" s="2">
-        <v>5.610661E-05</v>
+        <v>5.982589E-05</v>
       </c>
       <c r="C119" s="2">
-        <v>5.624821E-05</v>
+        <v>5.994993E-05</v>
       </c>
       <c r="D119" s="2">
-        <v>9.324548E-06</v>
+        <v>1.114156E-05</v>
       </c>
       <c r="E119" s="2">
-        <v>0.0001080867</v>
+        <v>0.0001099091</v>
       </c>
     </row>
     <row r="120">
@@ -2207,16 +2207,16 @@
         <v>21.5</v>
       </c>
       <c r="B120" s="2">
-        <v>5.600738E-05</v>
+        <v>5.972387E-05</v>
       </c>
       <c r="C120" s="2">
-        <v>5.614743E-05</v>
+        <v>5.984604E-05</v>
       </c>
       <c r="D120" s="2">
-        <v>9.38284E-06</v>
+        <v>1.121245E-05</v>
       </c>
       <c r="E120" s="2">
-        <v>0.0001078913</v>
+        <v>0.000109717</v>
       </c>
     </row>
     <row r="121">
@@ -2224,16 +2224,16 @@
         <v>21.75</v>
       </c>
       <c r="B121" s="2">
-        <v>5.590995E-05</v>
+        <v>5.962377E-05</v>
       </c>
       <c r="C121" s="2">
-        <v>5.604846E-05</v>
+        <v>5.97441E-05</v>
       </c>
       <c r="D121" s="2">
-        <v>9.441008E-06</v>
+        <v>1.128319E-05</v>
       </c>
       <c r="E121" s="2">
-        <v>0.0001076995</v>
+        <v>0.0001095285</v>
       </c>
     </row>
     <row r="122">
@@ -2241,16 +2241,16 @@
         <v>22</v>
       </c>
       <c r="B122" s="2">
-        <v>5.581427E-05</v>
+        <v>5.952556E-05</v>
       </c>
       <c r="C122" s="2">
-        <v>5.595126E-05</v>
+        <v>5.964407E-05</v>
       </c>
       <c r="D122" s="2">
-        <v>9.499054E-06</v>
+        <v>1.135378E-05</v>
       </c>
       <c r="E122" s="2">
-        <v>0.000107511</v>
+        <v>0.0001093435</v>
       </c>
     </row>
     <row r="123">
@@ -2258,16 +2258,16 @@
         <v>22.25</v>
       </c>
       <c r="B123" s="2">
-        <v>5.572031E-05</v>
+        <v>5.942917E-05</v>
       </c>
       <c r="C123" s="2">
-        <v>5.585579E-05</v>
+        <v>5.954591E-05</v>
       </c>
       <c r="D123" s="2">
-        <v>9.556978E-06</v>
+        <v>1.142422E-05</v>
       </c>
       <c r="E123" s="2">
-        <v>0.000107326</v>
+        <v>0.0001091619</v>
       </c>
     </row>
     <row r="124">
@@ -2275,16 +2275,16 @@
         <v>22.5</v>
       </c>
       <c r="B124" s="2">
-        <v>5.562802E-05</v>
+        <v>5.933462E-05</v>
       </c>
       <c r="C124" s="2">
-        <v>5.576202E-05</v>
+        <v>5.944961E-05</v>
       </c>
       <c r="D124" s="2">
-        <v>9.614783E-06</v>
+        <v>1.149451E-05</v>
       </c>
       <c r="E124" s="2">
-        <v>0.0001071442</v>
+        <v>0.0001089838</v>
       </c>
     </row>
     <row r="125">
@@ -2292,16 +2292,16 @@
         <v>22.75</v>
       </c>
       <c r="B125" s="2">
-        <v>5.553738E-05</v>
+        <v>5.924183E-05</v>
       </c>
       <c r="C125" s="2">
-        <v>5.566991E-05</v>
+        <v>5.935509E-05</v>
       </c>
       <c r="D125" s="2">
-        <v>9.672471E-06</v>
+        <v>1.156466E-05</v>
       </c>
       <c r="E125" s="2">
-        <v>0.0001069657</v>
+        <v>0.000108809</v>
       </c>
     </row>
     <row r="126">
@@ -2309,16 +2309,16 @@
         <v>23</v>
       </c>
       <c r="B126" s="2">
-        <v>5.544833E-05</v>
+        <v>5.915079E-05</v>
       </c>
       <c r="C126" s="2">
-        <v>5.55794E-05</v>
+        <v>5.926235E-05</v>
       </c>
       <c r="D126" s="2">
-        <v>9.730044E-06</v>
+        <v>1.163467E-05</v>
       </c>
       <c r="E126" s="2">
-        <v>0.0001067903</v>
+        <v>0.0001086374</v>
       </c>
     </row>
     <row r="127">
@@ -2326,16 +2326,16 @@
         <v>23.25</v>
       </c>
       <c r="B127" s="2">
-        <v>5.536083E-05</v>
+        <v>5.906144E-05</v>
       </c>
       <c r="C127" s="2">
-        <v>5.549048E-05</v>
+        <v>5.917134E-05</v>
       </c>
       <c r="D127" s="2">
-        <v>9.787504E-06</v>
+        <v>1.170454E-05</v>
       </c>
       <c r="E127" s="2">
-        <v>0.0001066179</v>
+        <v>0.0001084691</v>
       </c>
     </row>
     <row r="128">
@@ -2343,16 +2343,16 @@
         <v>23.5</v>
       </c>
       <c r="B128" s="2">
-        <v>5.527489E-05</v>
+        <v>5.897377E-05</v>
       </c>
       <c r="C128" s="2">
-        <v>5.540312E-05</v>
+        <v>5.908203E-05</v>
       </c>
       <c r="D128" s="2">
-        <v>9.844851E-06</v>
+        <v>1.177427E-05</v>
       </c>
       <c r="E128" s="2">
-        <v>0.0001064486</v>
+        <v>0.0001083039</v>
       </c>
     </row>
     <row r="129">
@@ -2360,16 +2360,16 @@
         <v>23.75</v>
       </c>
       <c r="B129" s="2">
-        <v>5.519045E-05</v>
+        <v>5.888774E-05</v>
       </c>
       <c r="C129" s="2">
-        <v>5.531729E-05</v>
+        <v>5.899438E-05</v>
       </c>
       <c r="D129" s="2">
-        <v>9.902088E-06</v>
+        <v>1.184387E-05</v>
       </c>
       <c r="E129" s="2">
-        <v>0.0001062822</v>
+        <v>0.0001081419</v>
       </c>
     </row>
     <row r="130">
@@ -2377,16 +2377,16 @@
         <v>24</v>
       </c>
       <c r="B130" s="2">
-        <v>5.510748E-05</v>
+        <v>5.880333E-05</v>
       </c>
       <c r="C130" s="2">
-        <v>5.523294E-05</v>
+        <v>5.890839E-05</v>
       </c>
       <c r="D130" s="2">
-        <v>9.959217E-06</v>
+        <v>1.191333E-05</v>
       </c>
       <c r="E130" s="2">
-        <v>0.0001061187</v>
+        <v>0.0001079828</v>
       </c>
     </row>
   </sheetData>
@@ -2401,7 +2401,7 @@
   <cols>
     <col min="1" max="1" width="23.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.55" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.05" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2427,7 +2427,7 @@
         <v>10</v>
       </c>
       <c r="C2" s="2">
-        <v>3870.3773021698</v>
+        <v>3805.67097663879</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -2441,7 +2441,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="2">
-        <v>4167.89722442627</v>
+        <v>4072.22270965576</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>11</v>
@@ -2455,7 +2455,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="2">
-        <v>0.41803898056969</v>
+        <v>0.389414752135053</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>14</v>
@@ -2469,7 +2469,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="2">
-        <v>6633.56431237184</v>
+        <v>6313.13484274689</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>11</v>
@@ -2486,10 +2486,10 @@
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="68.55" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.85" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="68.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2514,16 +2514,16 @@
         <v>20</v>
       </c>
       <c r="B2" s="2">
-        <v>0.673915386199951</v>
+        <v>0.74267053604126</v>
       </c>
       <c r="C2" s="2">
         <v>0</v>
       </c>
       <c r="D2" s="2">
-        <v>1.29800271987915</v>
+        <v>1.36377000808716</v>
       </c>
       <c r="E2" s="2">
-        <v>0.684157013893127</v>
+        <v>0.755667507648468</v>
       </c>
     </row>
     <row r="3">
@@ -2531,16 +2531,16 @@
         <v>21</v>
       </c>
       <c r="B3" s="2">
-        <v>2356312011718.75</v>
+        <v>2523789062500</v>
       </c>
       <c r="C3" s="2">
         <v>0</v>
       </c>
       <c r="D3" s="2">
-        <v>4538402832031.25</v>
+        <v>4634447753906.25</v>
       </c>
       <c r="E3" s="2">
-        <v>2392121582031.25</v>
+        <v>2567956054687.5</v>
       </c>
     </row>
     <row r="4">
@@ -2548,16 +2548,16 @@
         <v>22</v>
       </c>
       <c r="B4" s="2">
-        <v>0.1309754550457</v>
+        <v>0.136948943138123</v>
       </c>
       <c r="C4" s="2">
-        <v>0.0098585095256567</v>
+        <v>0.0117086069658399</v>
       </c>
       <c r="D4" s="2">
-        <v>0.263966649770737</v>
+        <v>0.263195216655731</v>
       </c>
       <c r="E4" s="2">
-        <v>0.134729012846947</v>
+        <v>0.140744015574455</v>
       </c>
     </row>
     <row r="5">
@@ -2565,16 +2565,16 @@
         <v>23</v>
       </c>
       <c r="B5" s="2">
-        <v>457949249267.578</v>
+        <v>465388397216.797</v>
       </c>
       <c r="C5" s="2">
-        <v>34469795227.0508</v>
+        <v>39788913726.8066</v>
       </c>
       <c r="D5" s="2">
-        <v>922946472167.969</v>
+        <v>894406250000</v>
       </c>
       <c r="E5" s="2">
-        <v>471073394775.391</v>
+        <v>478285064697.266</v>
       </c>
     </row>
     <row r="6">
@@ -2582,16 +2582,16 @@
         <v>24</v>
       </c>
       <c r="B6" s="2">
-        <v>0.00116683600936085</v>
+        <v>0.00118439120706171</v>
       </c>
       <c r="C6" s="2">
-        <v>9.95921709545655E-06</v>
+        <v>1.19133346743183E-05</v>
       </c>
       <c r="D6" s="2">
-        <v>0.00191633054055274</v>
+        <v>0.00194960727822036</v>
       </c>
       <c r="E6" s="2">
-        <v>0.00149069831240922</v>
+        <v>0.0015145834768191</v>
       </c>
     </row>
     <row r="7">
@@ -2599,16 +2599,16 @@
         <v>25</v>
       </c>
       <c r="B7" s="2">
-        <v>4079784.87014771</v>
+        <v>4024871.82617188</v>
       </c>
       <c r="C7" s="2">
-        <v>34821.9163715839</v>
+        <v>40484.6332967281</v>
       </c>
       <c r="D7" s="2">
-        <v>6700356.00662231</v>
+        <v>6625276.56555176</v>
       </c>
       <c r="E7" s="2">
-        <v>5212153.43475342</v>
+        <v>5146951.67541504</v>
       </c>
     </row>
     <row r="8">
@@ -2616,16 +2616,16 @@
         <v>26</v>
       </c>
       <c r="B8" s="2">
-        <v>5.52329438505694E-05</v>
+        <v>5.89083865634166E-05</v>
       </c>
       <c r="C8" s="2">
-        <v>9.95921709545655E-06</v>
+        <v>1.19133346743183E-05</v>
       </c>
       <c r="D8" s="2">
-        <v>0.000106118721305393</v>
+        <v>0.000107982814370189</v>
       </c>
       <c r="E8" s="2">
-        <v>5.51074808754493E-05</v>
+        <v>5.88033326494042E-05</v>
       </c>
     </row>
     <row r="9">
@@ -2633,16 +2633,16 @@
         <v>27</v>
       </c>
       <c r="B9" s="2">
-        <v>0.42439199751243</v>
+        <v>0.396229617763311</v>
       </c>
       <c r="C9" s="2" t="e">
         <v>#DIV/0!</v>
       </c>
       <c r="D9" s="2">
-        <v>0.220341826207004</v>
+        <v>0.215775435208343</v>
       </c>
       <c r="E9" s="2">
-        <v>0.41803898056969</v>
+        <v>0.389414752135053</v>
       </c>
     </row>
     <row r="10">
@@ -2650,16 +2650,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="2">
-        <v>0.805649995803833</v>
+        <v>0.815599322319031</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2">
-        <v>0.796636283397675</v>
+        <v>0.807009100914001</v>
       </c>
       <c r="E10" s="2">
-        <v>0.803072988986969</v>
+        <v>0.813748717308044</v>
       </c>
     </row>
     <row r="11">
@@ -2667,16 +2667,16 @@
         <v>30</v>
       </c>
       <c r="B11" s="2">
-        <v>152.936165364583</v>
+        <v>160.893701171875</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2">
-        <v>150.109114583333</v>
+        <v>158.006770833333</v>
       </c>
       <c r="E11" s="2">
-        <v>154.306884765625</v>
+        <v>162.879931640625</v>
       </c>
     </row>
     <row r="12">
@@ -2701,16 +2701,16 @@
         <v>32</v>
       </c>
       <c r="B13" s="2">
-        <v>113.560628255208</v>
+        <v>118.787337239583</v>
       </c>
       <c r="C13" s="2">
-        <v>-30.1221130371094</v>
+        <v>-29.6323994954427</v>
       </c>
       <c r="D13" s="2">
-        <v>112.568758138021</v>
+        <v>117.744099934896</v>
       </c>
       <c r="E13" s="2">
-        <v>115.179305013021</v>
+        <v>120.807340494792</v>
       </c>
     </row>
     <row r="14">
@@ -2718,16 +2718,16 @@
         <v>33</v>
       </c>
       <c r="B14" s="2">
-        <v>4171.77391052246</v>
+        <v>4074.20492172241</v>
       </c>
       <c r="C14" s="2" t="e">
         <v>#DIV/0!</v>
       </c>
       <c r="D14" s="2">
-        <v>2147.04251289368</v>
+        <v>2199.21112060547</v>
       </c>
       <c r="E14" s="2">
-        <v>4167.89722442627</v>
+        <v>4072.22270965576</v>
       </c>
     </row>
     <row r="15">
@@ -2735,16 +2735,16 @@
         <v>34</v>
       </c>
       <c r="B15" s="2">
-        <v>3894.29330825806</v>
+        <v>3825.05106925964</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="2">
-        <v>1984.51900482178</v>
+        <v>2045.63856124878</v>
       </c>
       <c r="E15" s="2">
-        <v>3870.3773021698</v>
+        <v>3805.67097663879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>